<commit_message>
Tufts calibration updates 1/21
</commit_message>
<xml_diff>
--- a/InputData/elec/SYC/Start Year Capacities.xlsx
+++ b/InputData/elec/SYC/Start Year Capacities.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/elec/SYC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{380224DD-DC44-514D-979E-CEF6ADAF5166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2055A71B-BB57-D649-963A-9796E1BEF296}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4300" yWindow="780" windowWidth="29900" windowHeight="21360" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -61991,7 +61991,8 @@
         <v>0</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <f>Capacity!B32</f>
+        <v>31000</v>
       </c>
       <c r="G2" s="78"/>
     </row>

</xml_diff>

<commit_message>
Tufts elec calibration BECF, BFPaT, and SYC
</commit_message>
<xml_diff>
--- a/InputData/elec/SYC/Start Year Capacities.xlsx
+++ b/InputData/elec/SYC/Start Year Capacities.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/elec/SYC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2055A71B-BB57-D649-963A-9796E1BEF296}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D56ADC6D-F093-8B41-857A-634C7BA5E94D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4300" yWindow="780" windowWidth="29900" windowHeight="21360" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -91,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="100">
   <si>
     <t>SYC Start Year Electricity Generation Capacity</t>
   </si>
@@ -758,6 +758,12 @@
   <si>
     <t>https://www.iea.org/data-and-statistics/charts/capacity-of-coal-fired-power-plants-in-southeast-asia-2019</t>
   </si>
+  <si>
+    <t>CREA</t>
+  </si>
+  <si>
+    <t>https://energyandcleanair.org/wp/wp-content/uploads/2023/03/CREA_Trend-Asia_EN_Ambiguities-versus-Ambition.pdf</t>
+  </si>
 </sst>
 </file>
 
@@ -1230,7 +1236,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1465,6 +1471,8 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1474,6 +1482,7 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1690,7 +1699,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B1002"/>
+  <dimension ref="A1:B1010"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.6640625" customWidth="1"/>
@@ -1753,35 +1762,47 @@
       </c>
     </row>
     <row r="12" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="13" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
+    <row r="13" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="14" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
-        <v>8</v>
+      <c r="B14" s="1" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="17" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
+      <c r="B15" s="4">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="91" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="18" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="19" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="20" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="21" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="22" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="23" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="21" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
     <row r="24" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="25" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="25" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
     <row r="26" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="27" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="28" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -2759,9 +2780,18 @@
     <row r="1000" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1001" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1002" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1003" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1004" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1005" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1006" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1007" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1008" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1009" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1010" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B11" r:id="rId1" xr:uid="{AE0DB459-E9B4-244D-A80B-99CD303D14E8}"/>
+    <hyperlink ref="B16" r:id="rId2" xr:uid="{2DE2A41A-7EA7-5543-8843-E077D7C000A1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>
@@ -4056,24 +4086,24 @@
       <c r="Z27" s="6"/>
     </row>
     <row r="28" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="84" t="s">
+      <c r="A28" s="86" t="s">
         <v>27</v>
       </c>
-      <c r="B28" s="85"/>
-      <c r="C28" s="85"/>
-      <c r="D28" s="85"/>
-      <c r="E28" s="85"/>
-      <c r="F28" s="85"/>
-      <c r="G28" s="86"/>
+      <c r="B28" s="87"/>
+      <c r="C28" s="87"/>
+      <c r="D28" s="87"/>
+      <c r="E28" s="87"/>
+      <c r="F28" s="87"/>
+      <c r="G28" s="88"/>
       <c r="H28" s="31"/>
       <c r="I28" s="31"/>
-      <c r="J28" s="87" t="s">
+      <c r="J28" s="89" t="s">
         <v>28</v>
       </c>
-      <c r="K28" s="85"/>
-      <c r="L28" s="85"/>
-      <c r="M28" s="85"/>
-      <c r="N28" s="88"/>
+      <c r="K28" s="87"/>
+      <c r="L28" s="87"/>
+      <c r="M28" s="87"/>
+      <c r="N28" s="90"/>
       <c r="O28" s="6"/>
       <c r="P28" s="6"/>
       <c r="Q28" s="6"/>
@@ -31972,7 +32002,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AA1004"/>
+  <dimension ref="A1:AA1003"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.5" customWidth="1"/>
@@ -33723,7 +33753,7 @@
         <v>94</v>
       </c>
       <c r="B32" s="6">
-        <v>31000</v>
+        <v>12000</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
@@ -33785,8 +33815,13 @@
       <c r="AA33" s="6"/>
     </row>
     <row r="34" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="6"/>
-      <c r="B34" s="6"/>
+      <c r="A34" s="60" t="s">
+        <v>48</v>
+      </c>
+      <c r="B34" s="75">
+        <f>D24+E24+H24</f>
+        <v>19860.009999999998</v>
+      </c>
       <c r="C34" s="6"/>
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
@@ -61914,35 +61949,6 @@
       <c r="Z1003" s="6"/>
       <c r="AA1003" s="6"/>
     </row>
-    <row r="1004" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1004" s="6"/>
-      <c r="B1004" s="6"/>
-      <c r="C1004" s="6"/>
-      <c r="D1004" s="6"/>
-      <c r="E1004" s="6"/>
-      <c r="F1004" s="6"/>
-      <c r="G1004" s="6"/>
-      <c r="H1004" s="6"/>
-      <c r="I1004" s="6"/>
-      <c r="J1004" s="6"/>
-      <c r="K1004" s="6"/>
-      <c r="L1004" s="6"/>
-      <c r="M1004" s="6"/>
-      <c r="N1004" s="6"/>
-      <c r="O1004" s="6"/>
-      <c r="P1004" s="6"/>
-      <c r="Q1004" s="6"/>
-      <c r="R1004" s="6"/>
-      <c r="S1004" s="6"/>
-      <c r="T1004" s="6"/>
-      <c r="U1004" s="6"/>
-      <c r="V1004" s="6"/>
-      <c r="W1004" s="6"/>
-      <c r="X1004" s="6"/>
-      <c r="Y1004" s="6"/>
-      <c r="Z1004" s="6"/>
-      <c r="AA1004" s="6"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>
@@ -61983,16 +61989,14 @@
       <c r="A2" s="78" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="77">
-        <f>SUMIF(Capacity!4:4, A2, Capacity!24:24)</f>
-        <v>34737.17</v>
+      <c r="B2" s="84">
+        <v>34600</v>
       </c>
       <c r="C2" s="77">
         <v>0</v>
       </c>
       <c r="D2">
-        <f>Capacity!B32</f>
-        <v>31000</v>
+        <v>3600</v>
       </c>
       <c r="G2" s="78"/>
     </row>
@@ -62000,24 +62004,24 @@
       <c r="A3" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B3" s="77">
-        <v>4984</v>
+      <c r="B3" s="84">
+        <f>Capacity!B34</f>
+        <v>19860.009999999998</v>
       </c>
       <c r="C3" s="77">
-        <f>SUMIF(Capacity!$B$4:$P$4,A3,Capacity!$B$24:$P$24)</f>
-        <v>5348.44</v>
+        <v>0</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
+      <c r="F3" s="85"/>
       <c r="G3" s="78"/>
     </row>
     <row r="4" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B4" s="77">
-        <f>SUMIF(Capacity!6:6, A4, Capacity!26:26)</f>
+      <c r="B4" s="84">
         <v>0</v>
       </c>
       <c r="C4" s="77">
@@ -62033,9 +62037,8 @@
       <c r="A5" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B5" s="77">
-        <f>SUMIF(Capacity!$4:$4, A5, Capacity!24:24)</f>
-        <v>5031.1500000000005</v>
+      <c r="B5" s="84">
+        <v>5980</v>
       </c>
       <c r="C5" s="77">
         <v>0</v>
@@ -62049,9 +62052,8 @@
       <c r="A6" s="78" t="s">
         <v>69</v>
       </c>
-      <c r="B6" s="77">
-        <f>SUMIF(Capacity!$4:$4, A6, Capacity!$24:$24)</f>
-        <v>153.83000000000001</v>
+      <c r="B6" s="84">
+        <v>150</v>
       </c>
       <c r="C6" s="77">
         <v>0</v>
@@ -62065,9 +62067,8 @@
       <c r="A7" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B7" s="77">
-        <f>SUMIF(Capacity!$4:$4, A7, Capacity!$24:$24)</f>
-        <v>105.03</v>
+      <c r="B7" s="84">
+        <v>150</v>
       </c>
       <c r="C7" s="77">
         <v>0</v>
@@ -62081,8 +62082,7 @@
       <c r="A8" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B8" s="77">
-        <f>SUMIF(Capacity!$4:$4, A8, Capacity!$24:$24)</f>
+      <c r="B8" s="84">
         <v>0</v>
       </c>
       <c r="C8" s="77">
@@ -62098,9 +62098,8 @@
       <c r="A9" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B9" s="77">
-        <f>SUMIF(Capacity!$4:$4, A9, Capacity!$24:$24)</f>
-        <v>147.02000000000001</v>
+      <c r="B9" s="84">
+        <v>1880</v>
       </c>
       <c r="C9" s="77">
         <v>0</v>
@@ -62114,9 +62113,8 @@
       <c r="A10" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B10" s="77">
-        <f>SUMIF(Capacity!$4:$4, A10, Capacity!$24:$24)</f>
-        <v>2130.6999999999998</v>
+      <c r="B10" s="84">
+        <v>2140</v>
       </c>
       <c r="C10" s="77">
         <v>0</v>
@@ -62130,8 +62128,8 @@
       <c r="A11" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B11" s="77">
-        <f>SUMIF(Capacity!$4:$4, A11, Capacity!$24:$24)</f>
+      <c r="B11" s="84">
+        <f>Capacity!G24</f>
         <v>4779.68</v>
       </c>
       <c r="C11" s="77">
@@ -62146,9 +62144,8 @@
       <c r="A12" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B12" s="77">
-        <f>SUMIF(Capacity!$4:$4, A12, Capacity!$24:$24)</f>
-        <v>2842.03</v>
+      <c r="B12" s="84">
+        <v>0</v>
       </c>
       <c r="C12" s="77">
         <v>0</v>
@@ -62162,9 +62159,8 @@
       <c r="A13" s="79" t="s">
         <v>72</v>
       </c>
-      <c r="B13" s="77">
-        <f>SUMIF(Capacity!$4:$4, A13, Capacity!$24:$24)</f>
-        <v>42.15</v>
+      <c r="B13" s="84">
+        <v>0</v>
       </c>
       <c r="C13" s="77">
         <v>0</v>
@@ -62178,8 +62174,7 @@
       <c r="A14" s="78" t="s">
         <v>88</v>
       </c>
-      <c r="B14" s="77">
-        <f>SUMIF(Capacity!$4:$4, A14, Capacity!$24:$24)</f>
+      <c r="B14" s="84">
         <v>0</v>
       </c>
       <c r="C14" s="77">
@@ -62194,8 +62189,7 @@
       <c r="A15" s="78" t="s">
         <v>89</v>
       </c>
-      <c r="B15" s="77">
-        <f>SUMIF(Capacity!$4:$4, A15, Capacity!$24:$24)</f>
+      <c r="B15" s="84">
         <v>0</v>
       </c>
       <c r="C15" s="77">
@@ -62210,8 +62204,7 @@
       <c r="A16" s="78" t="s">
         <v>90</v>
       </c>
-      <c r="B16" s="77">
-        <f>SUMIF(Capacity!$4:$4, A16, Capacity!$24:$24)</f>
+      <c r="B16" s="84">
         <v>0</v>
       </c>
       <c r="C16" s="77">
@@ -62226,8 +62219,7 @@
       <c r="A17" s="78" t="s">
         <v>91</v>
       </c>
-      <c r="B17" s="77">
-        <f>SUMIF(Capacity!$4:$4, A17, Capacity!$24:$24)</f>
+      <c r="B17" s="84">
         <v>0</v>
       </c>
       <c r="C17" s="77">
@@ -62242,9 +62234,8 @@
       <c r="A18" s="78" t="s">
         <v>71</v>
       </c>
-      <c r="B18" s="77">
-        <f>SUMIF(Capacity!$4:$4, A18, Capacity!$24:$24)</f>
-        <v>15.65</v>
+      <c r="B18" s="84">
+        <v>0</v>
       </c>
       <c r="C18" s="77">
         <v>0</v>

</xml_diff>